<commit_message>
using successresponse schema for blog deletion
</commit_message>
<xml_diff>
--- a/database_export.xlsx
+++ b/database_export.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N15"/>
+  <dimension ref="A1:Q16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -446,12 +446,15 @@
     <col width="9" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="114" customWidth="1" min="9" max="9"/>
-    <col width="115" customWidth="1" min="10" max="10"/>
-    <col width="114" customWidth="1" min="11" max="11"/>
+    <col width="137" customWidth="1" min="9" max="9"/>
+    <col width="138" customWidth="1" min="10" max="10"/>
+    <col width="137" customWidth="1" min="11" max="11"/>
     <col width="763" customWidth="1" min="12" max="12"/>
     <col width="595" customWidth="1" min="13" max="13"/>
     <col width="84" customWidth="1" min="14" max="14"/>
+    <col width="69" customWidth="1" min="15" max="15"/>
+    <col width="70" customWidth="1" min="16" max="16"/>
+    <col width="69" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -525,6 +528,21 @@
           <t>slug</t>
         </is>
       </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>image_public_id_small</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>image_public_id_medium</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>image_public_id_large</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -587,6 +605,9 @@
           <t>hello-ai</t>
         </is>
       </c>
+      <c r="O2" s="2" t="n"/>
+      <c r="P2" s="2" t="n"/>
+      <c r="Q2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -857,6 +878,9 @@
           <t>ai-trial</t>
         </is>
       </c>
+      <c r="O3" s="2" t="n"/>
+      <c r="P3" s="2" t="n"/>
+      <c r="Q3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -1255,6 +1279,9 @@
           <t>owasp-top-10-tryhackme</t>
         </is>
       </c>
+      <c r="O4" s="2" t="n"/>
+      <c r="P4" s="2" t="n"/>
+      <c r="Q4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -1760,6 +1787,9 @@
           <t>wreath-tryhackme</t>
         </is>
       </c>
+      <c r="O5" s="2" t="n"/>
+      <c r="P5" s="2" t="n"/>
+      <c r="Q5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -1853,6 +1883,9 @@
           <t>embracing-the-power-of-small-habits</t>
         </is>
       </c>
+      <c r="O6" s="2" t="n"/>
+      <c r="P6" s="2" t="n"/>
+      <c r="Q6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -1991,6 +2024,9 @@
           <t>the-psychology-of-color-how-colors-influence-our-emotions-decisions-and-perception</t>
         </is>
       </c>
+      <c r="O7" s="2" t="n"/>
+      <c r="P7" s="2" t="n"/>
+      <c r="Q7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -2451,6 +2487,9 @@
           <t>snort-tryhackme</t>
         </is>
       </c>
+      <c r="O8" s="2" t="n"/>
+      <c r="P8" s="2" t="n"/>
+      <c r="Q8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -2595,6 +2634,9 @@
           <t>racetrack-bank-tryhackme</t>
         </is>
       </c>
+      <c r="O9" s="2" t="n"/>
+      <c r="P9" s="2" t="n"/>
+      <c r="Q9" s="2" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -2658,6 +2700,9 @@
           <t>magical-image-gallery-hacker101</t>
         </is>
       </c>
+      <c r="O10" s="2" t="n"/>
+      <c r="P10" s="2" t="n"/>
+      <c r="Q10" s="2" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -2721,6 +2766,9 @@
           <t>just-testing</t>
         </is>
       </c>
+      <c r="O11" s="2" t="n"/>
+      <c r="P11" s="2" t="n"/>
+      <c r="Q11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -2831,6 +2879,9 @@
           <t>the-magic-of-night-photography-capturing-the-unseen</t>
         </is>
       </c>
+      <c r="O12" s="2" t="n"/>
+      <c r="P12" s="2" t="n"/>
+      <c r="Q12" s="2" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -2927,6 +2978,9 @@
           <t>the-rise-of-plant-based-diets-a-healthier-future</t>
         </is>
       </c>
+      <c r="O13" s="2" t="n"/>
+      <c r="P13" s="2" t="n"/>
+      <c r="Q13" s="2" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -3032,6 +3086,9 @@
           <t>quantum-computing</t>
         </is>
       </c>
+      <c r="O14" s="2" t="n"/>
+      <c r="P14" s="2" t="n"/>
+      <c r="Q14" s="2" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -3205,6 +3262,87 @@
       <c r="N15" s="2" t="inlineStr">
         <is>
           <t>exploiting-active-directory-tryhackme</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="n"/>
+      <c r="P15" s="2" t="n"/>
+      <c r="Q15" s="2" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Cloudinary Upload test, The Future of Cloud Image Uploading</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;In today&amp;rsquo;s digital age, cloud image uploading has revolutionized how we store, share, and manage visual content. Whether you're a photographer, a social media enthusiast, or a business owner, cloud-based solutions offer unparalleled convenience and efficiency. Platforms like Google Drive, AWS S3, and Cloudinary allow users to upload images seamlessly, eliminating the need for physical storage devices and reducing the risk of data loss.&lt;/p&gt;
+&lt;p&gt;One of the biggest advantages of cloud image uploading is accessibility. Your images are available anytime, anywhere, as long as you have an internet connection. This makes collaboration effortless, enabling teams to share and edit files in real time. Additionally, cloud services often provide advanced features like automatic backups, version control, and AI-powered image optimization, ensuring your files are both secure and high-quality.&lt;/p&gt;
+&lt;p&gt;Security is another key benefit. Reputable cloud providers use encryption and multi-factor authentication to protect your data from unauthorized access. Scalability is equally important&amp;mdash;cloud storage can grow with your needs, allowing you to store thousands of images without worrying about running out of space.&lt;/p&gt;
+&lt;p&gt;However, it&amp;rsquo;s essential to choose a reliable provider and understand their pricing models to avoid unexpected costs. With the right approach, cloud image uploading can streamline your workflow, enhance collaboration, and safeguard your memories or business assets for years to come. Embrace the cloud&amp;mdash;it&amp;rsquo;s the future of image management!&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Cloud Storage</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G16" s="3" t="n">
+        <v>45664.33653908136</v>
+      </c>
+      <c r="H16" s="3" t="n"/>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dbdrbl0jt/image/upload/v1736237078/Cloudinary_Upload_test%2C_The_Future_of_Cloud_Image_Uploading_5_small.png</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dbdrbl0jt/image/upload/v1736237079/Cloudinary_Upload_test%2C_The_Future_of_Cloud_Image_Uploading_5_medium.png</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>https://res.cloudinary.com/dbdrbl0jt/image/upload/v1736237079/Cloudinary_Upload_test%2C_The_Future_of_Cloud_Image_Uploading_5_large.png</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>Cloud image uploading has transformed visual content management, offering convenience, efficiency, and accessibility. Platforms like Google Drive and AWS S3 provide seamless uploads, eliminating physical storage and reducing data loss risk. Images are accessible anytime, anywhere, facilitating real-time collaboration. Advanced features like automatic backups and AI optimization ensure file security and quality. Reputable providers use encryption for protection, and scalability accommodates growing storage needs. Choosing a reliable provider and understanding pricing models is crucial. Cloud image uploading streamlines workflows, enhances collaboration, and safeguards assets, embodying the future of image management.</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>Cloud image uploading offers unparalleled convenience, accessibility, and security for storing and managing visual content. With features like automatic backups, AI-powered optimization, encryption, and scalability, cloud-based solutions streamline workflow, enhance collaboration, and safeguard memories or business assets.</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>cloudinary-upload-test-the-future-of-cloud-image-uploading</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>Cloudinary_Upload_test,_The_Future_of_Cloud_Image_Uploading_5_small</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>Cloudinary_Upload_test,_The_Future_of_Cloud_Image_Uploading_5_medium</t>
+        </is>
+      </c>
+      <c r="Q16" s="2" t="inlineStr">
+        <is>
+          <t>Cloudinary_Upload_test,_The_Future_of_Cloud_Image_Uploading_5_large</t>
         </is>
       </c>
     </row>

</xml_diff>